<commit_message>
Add editor draft and publisher review workflow across admin menus.
Editors create and submit drafts; publishers publish or reject with notes (except Rehab Centers, which stays shared add/edit/archive). Inbox notifications deep-link to each module, and public APIs only expose published content.
</commit_message>
<xml_diff>
--- a/docs/uat-admin-test-scripts/DAPE-MA-ADMIN-UAT-TEST-SCRIPTS.xlsx
+++ b/docs/uat-admin-test-scripts/DAPE-MA-ADMIN-UAT-TEST-SCRIPTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/XAMPP/xamppfiles/htdocs/DAPE-MA/dape-ma-laravel/docs/uat-admin-test-scripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DCAA901-AE1D-DC4A-A2B4-538BA00040AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F106E760-3599-904F-AF6D-9A45E8E2D8D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="20140" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="20140" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="832">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1159" uniqueCount="832">
   <si>
     <t>DAPE-MA – Admin Control Panel User Acceptance Test Scripts</t>
   </si>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="C5" s="4">
         <f>COUNTIF(Publisher!J2:J12,"Pass")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D5" s="4">
         <f>COUNTIF(Publisher!J2:J12,"Fail")</f>
@@ -3518,11 +3518,11 @@
       </c>
       <c r="F5" s="4">
         <f>B5-C5-D5-E5</f>
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G5" s="5">
         <f>IF(B5=0,0,C5/B5)</f>
-        <v>0</v>
+        <v>0.36363636363636365</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C6" s="4">
         <f>COUNTIF(Editor!J2:J10,"Pass")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D6" s="4">
         <f>COUNTIF(Editor!J2:J10,"Fail")</f>
@@ -3547,11 +3547,11 @@
       </c>
       <c r="F6" s="4">
         <f>B6-C6-D6-E6</f>
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G6" s="5">
         <f>IF(B6=0,0,C6/B6)</f>
-        <v>0</v>
+        <v>0.88888888888888884</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="C8" s="6">
         <f>SUM(C4:C7)</f>
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D8" s="6">
         <f>SUM(D4:D7)</f>
@@ -3605,11 +3605,11 @@
       </c>
       <c r="F8" s="6">
         <f>SUM(F4:F7)</f>
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="G8" s="7">
         <f>IF(B8=0,0,C8/B8)</f>
-        <v>5.4545454545454543E-2</v>
+        <v>0.16363636363636364</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -6197,6 +6197,9 @@
       <c r="H2" s="13" t="s">
         <v>611</v>
       </c>
+      <c r="J2" s="18" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="3" spans="1:14" ht="75" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
@@ -6223,6 +6226,9 @@
       <c r="H3" s="11" t="s">
         <v>616</v>
       </c>
+      <c r="J3" s="19" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="4" spans="1:14" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -6249,6 +6255,9 @@
       <c r="H4" s="13" t="s">
         <v>621</v>
       </c>
+      <c r="J4" s="18" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="5" spans="1:14" ht="30" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
@@ -6274,6 +6283,9 @@
       </c>
       <c r="H5" s="11" t="s">
         <v>626</v>
+      </c>
+      <c r="J5" s="19" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="30" x14ac:dyDescent="0.2">
@@ -6584,6 +6596,9 @@
       <c r="H2" s="13" t="s">
         <v>670</v>
       </c>
+      <c r="J2" s="18" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="3" spans="1:14" ht="60" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
@@ -6610,6 +6625,9 @@
       <c r="H3" s="11" t="s">
         <v>675</v>
       </c>
+      <c r="J3" s="19" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="4" spans="1:14" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -6636,6 +6654,9 @@
       <c r="H4" s="13" t="s">
         <v>680</v>
       </c>
+      <c r="J4" s="18" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="5" spans="1:14" ht="45" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
@@ -6662,6 +6683,9 @@
       <c r="H5" s="11" t="s">
         <v>686</v>
       </c>
+      <c r="J5" s="19" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="6" spans="1:14" ht="30" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="s">
@@ -6688,6 +6712,9 @@
       <c r="H6" s="13" t="s">
         <v>692</v>
       </c>
+      <c r="J6" s="18" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="7" spans="1:14" ht="30" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
@@ -6714,6 +6741,9 @@
       <c r="H7" s="11" t="s">
         <v>698</v>
       </c>
+      <c r="J7" s="19" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="8" spans="1:14" ht="30" x14ac:dyDescent="0.2">
       <c r="A8" s="13" t="s">
@@ -6740,6 +6770,9 @@
       <c r="H8" s="13" t="s">
         <v>703</v>
       </c>
+      <c r="J8" s="18" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
@@ -6765,6 +6798,9 @@
       </c>
       <c r="H9" s="11" t="s">
         <v>707</v>
+      </c>
+      <c r="J9" s="19" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">

</xml_diff>